<commit_message>
Daten bis 17. April
</commit_message>
<xml_diff>
--- a/result/szenarien_pivot.xlsx
+++ b/result/szenarien_pivot.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Info" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daten'!$A$1:$D$1081</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daten'!$A$1:$D$1273</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1081"/>
+  <dimension ref="A1:D1273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19945,8 +19945,3464 @@
         <v>2.11</v>
       </c>
     </row>
+    <row r="1082">
+      <c r="A1082" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B1082" s="2" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="C1082" s="3" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="D1082" s="3" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B1083" s="4" t="inlineStr">
+        <is>
+          <t>sz01</t>
+        </is>
+      </c>
+      <c r="C1083" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D1083" s="5" t="n">
+        <v>0.53</v>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B1084" s="2" t="inlineStr">
+        <is>
+          <t>sz02</t>
+        </is>
+      </c>
+      <c r="C1084" s="3" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="D1084" s="3" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B1085" s="4" t="inlineStr">
+        <is>
+          <t>sz03</t>
+        </is>
+      </c>
+      <c r="C1085" s="5" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="D1085" s="5" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B1086" s="2" t="inlineStr">
+        <is>
+          <t>sz04</t>
+        </is>
+      </c>
+      <c r="C1086" s="3" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D1086" s="3" t="n">
+        <v>1.63</v>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B1087" s="4" t="inlineStr">
+        <is>
+          <t>sz05</t>
+        </is>
+      </c>
+      <c r="C1087" s="5" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="D1087" s="5" t="n">
+        <v>1.86</v>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B1088" s="2" t="inlineStr">
+        <is>
+          <t>sz06</t>
+        </is>
+      </c>
+      <c r="C1088" s="3" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="D1088" s="3" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B1089" s="4" t="inlineStr">
+        <is>
+          <t>sz07</t>
+        </is>
+      </c>
+      <c r="C1089" s="5" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="D1089" s="5" t="n">
+        <v>0.46</v>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B1090" s="2" t="inlineStr">
+        <is>
+          <t>sz08</t>
+        </is>
+      </c>
+      <c r="C1090" s="3" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="D1090" s="3" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B1091" s="4" t="inlineStr">
+        <is>
+          <t>sz09</t>
+        </is>
+      </c>
+      <c r="C1091" s="5" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="D1091" s="5" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B1092" s="2" t="inlineStr">
+        <is>
+          <t>sz10</t>
+        </is>
+      </c>
+      <c r="C1092" s="3" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D1092" s="3" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B1093" s="4" t="inlineStr">
+        <is>
+          <t>sz11</t>
+        </is>
+      </c>
+      <c r="C1093" s="5" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="D1093" s="5" t="n">
+        <v>1.96</v>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B1094" s="2" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="C1094" s="3" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="D1094" s="3" t="n">
+        <v>-0.77</v>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B1095" s="4" t="inlineStr">
+        <is>
+          <t>sz01</t>
+        </is>
+      </c>
+      <c r="C1095" s="5" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="D1095" s="5" t="n">
+        <v>-0.04</v>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B1096" s="2" t="inlineStr">
+        <is>
+          <t>sz02</t>
+        </is>
+      </c>
+      <c r="C1096" s="3" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="D1096" s="3" t="n">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B1097" s="4" t="inlineStr">
+        <is>
+          <t>sz03</t>
+        </is>
+      </c>
+      <c r="C1097" s="5" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="D1097" s="5" t="n">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B1098" s="2" t="inlineStr">
+        <is>
+          <t>sz04</t>
+        </is>
+      </c>
+      <c r="C1098" s="3" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="D1098" s="3" t="n">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B1099" s="4" t="inlineStr">
+        <is>
+          <t>sz05</t>
+        </is>
+      </c>
+      <c r="C1099" s="5" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="D1099" s="5" t="n">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B1100" s="2" t="inlineStr">
+        <is>
+          <t>sz06</t>
+        </is>
+      </c>
+      <c r="C1100" s="3" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="D1100" s="3" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B1101" s="4" t="inlineStr">
+        <is>
+          <t>sz07</t>
+        </is>
+      </c>
+      <c r="C1101" s="5" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="D1101" s="5" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B1102" s="2" t="inlineStr">
+        <is>
+          <t>sz08</t>
+        </is>
+      </c>
+      <c r="C1102" s="3" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D1102" s="3" t="n">
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B1103" s="4" t="inlineStr">
+        <is>
+          <t>sz09</t>
+        </is>
+      </c>
+      <c r="C1103" s="5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D1103" s="5" t="n">
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B1104" s="2" t="inlineStr">
+        <is>
+          <t>sz10</t>
+        </is>
+      </c>
+      <c r="C1104" s="3" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D1104" s="3" t="n">
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B1105" s="4" t="inlineStr">
+        <is>
+          <t>sz11</t>
+        </is>
+      </c>
+      <c r="C1105" s="5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D1105" s="5" t="n">
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B1106" s="2" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="C1106" s="3" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="D1106" s="3" t="n">
+        <v>-0.47</v>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B1107" s="4" t="inlineStr">
+        <is>
+          <t>sz01</t>
+        </is>
+      </c>
+      <c r="C1107" s="5" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="D1107" s="5" t="n">
+        <v>-0.03</v>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B1108" s="2" t="inlineStr">
+        <is>
+          <t>sz02</t>
+        </is>
+      </c>
+      <c r="C1108" s="3" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="D1108" s="3" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B1109" s="4" t="inlineStr">
+        <is>
+          <t>sz03</t>
+        </is>
+      </c>
+      <c r="C1109" s="5" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="D1109" s="5" t="n">
+        <v>1.64</v>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B1110" s="2" t="inlineStr">
+        <is>
+          <t>sz04</t>
+        </is>
+      </c>
+      <c r="C1110" s="3" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="D1110" s="3" t="n">
+        <v>1.09</v>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B1111" s="4" t="inlineStr">
+        <is>
+          <t>sz05</t>
+        </is>
+      </c>
+      <c r="C1111" s="5" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="D1111" s="5" t="n">
+        <v>1.64</v>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B1112" s="2" t="inlineStr">
+        <is>
+          <t>sz06</t>
+        </is>
+      </c>
+      <c r="C1112" s="3" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="D1112" s="3" t="n">
+        <v>-0.23</v>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B1113" s="4" t="inlineStr">
+        <is>
+          <t>sz07</t>
+        </is>
+      </c>
+      <c r="C1113" s="5" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="D1113" s="5" t="n">
+        <v>-0.01</v>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B1114" s="2" t="inlineStr">
+        <is>
+          <t>sz08</t>
+        </is>
+      </c>
+      <c r="C1114" s="3" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="D1114" s="3" t="n">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B1115" s="4" t="inlineStr">
+        <is>
+          <t>sz09</t>
+        </is>
+      </c>
+      <c r="C1115" s="5" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="D1115" s="5" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B1116" s="2" t="inlineStr">
+        <is>
+          <t>sz10</t>
+        </is>
+      </c>
+      <c r="C1116" s="3" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="D1116" s="3" t="n">
+        <v>1.04</v>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B1117" s="4" t="inlineStr">
+        <is>
+          <t>sz11</t>
+        </is>
+      </c>
+      <c r="C1117" s="5" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="D1117" s="5" t="n">
+        <v>1.78</v>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B1118" s="2" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="C1118" s="3" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="D1118" s="3" t="n">
+        <v>-0.9</v>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B1119" s="4" t="inlineStr">
+        <is>
+          <t>sz01</t>
+        </is>
+      </c>
+      <c r="C1119" s="5" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="D1119" s="5" t="n">
+        <v>1.31</v>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B1120" s="2" t="inlineStr">
+        <is>
+          <t>sz02</t>
+        </is>
+      </c>
+      <c r="C1120" s="3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D1120" s="3" t="n">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B1121" s="4" t="inlineStr">
+        <is>
+          <t>sz03</t>
+        </is>
+      </c>
+      <c r="C1121" s="5" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D1121" s="5" t="n">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B1122" s="2" t="inlineStr">
+        <is>
+          <t>sz04</t>
+        </is>
+      </c>
+      <c r="C1122" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1122" s="3" t="n">
+        <v>1.84</v>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B1123" s="4" t="inlineStr">
+        <is>
+          <t>sz05</t>
+        </is>
+      </c>
+      <c r="C1123" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1123" s="5" t="n">
+        <v>1.84</v>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B1124" s="2" t="inlineStr">
+        <is>
+          <t>sz06</t>
+        </is>
+      </c>
+      <c r="C1124" s="3" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="D1124" s="3" t="n">
+        <v>-0.09</v>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B1125" s="4" t="inlineStr">
+        <is>
+          <t>sz07</t>
+        </is>
+      </c>
+      <c r="C1125" s="5" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="D1125" s="5" t="n">
+        <v>1.31</v>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B1126" s="2" t="inlineStr">
+        <is>
+          <t>sz08</t>
+        </is>
+      </c>
+      <c r="C1126" s="3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D1126" s="3" t="n">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B1127" s="4" t="inlineStr">
+        <is>
+          <t>sz09</t>
+        </is>
+      </c>
+      <c r="C1127" s="5" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D1127" s="5" t="n">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B1128" s="2" t="inlineStr">
+        <is>
+          <t>sz10</t>
+        </is>
+      </c>
+      <c r="C1128" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1128" s="3" t="n">
+        <v>1.84</v>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B1129" s="4" t="inlineStr">
+        <is>
+          <t>sz11</t>
+        </is>
+      </c>
+      <c r="C1129" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1129" s="5" t="n">
+        <v>1.84</v>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1130" s="2" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="C1130" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D1130" s="3" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1131" s="4" t="inlineStr">
+        <is>
+          <t>sz01</t>
+        </is>
+      </c>
+      <c r="C1131" s="5" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="D1131" s="5" t="n">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1132" s="2" t="inlineStr">
+        <is>
+          <t>sz02</t>
+        </is>
+      </c>
+      <c r="C1132" s="3" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="D1132" s="3" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1133" s="4" t="inlineStr">
+        <is>
+          <t>sz03</t>
+        </is>
+      </c>
+      <c r="C1133" s="5" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="D1133" s="5" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1134" s="2" t="inlineStr">
+        <is>
+          <t>sz04</t>
+        </is>
+      </c>
+      <c r="C1134" s="3" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="D1134" s="3" t="n">
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1135" s="4" t="inlineStr">
+        <is>
+          <t>sz05</t>
+        </is>
+      </c>
+      <c r="C1135" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1135" s="5" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1136" s="2" t="inlineStr">
+        <is>
+          <t>sz06</t>
+        </is>
+      </c>
+      <c r="C1136" s="3" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="D1136" s="3" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1137" s="4" t="inlineStr">
+        <is>
+          <t>sz07</t>
+        </is>
+      </c>
+      <c r="C1137" s="5" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="D1137" s="5" t="n">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1138" s="2" t="inlineStr">
+        <is>
+          <t>sz08</t>
+        </is>
+      </c>
+      <c r="C1138" s="3" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="D1138" s="3" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1139" s="4" t="inlineStr">
+        <is>
+          <t>sz09</t>
+        </is>
+      </c>
+      <c r="C1139" s="5" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="D1139" s="5" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1140" s="2" t="inlineStr">
+        <is>
+          <t>sz10</t>
+        </is>
+      </c>
+      <c r="C1140" s="3" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="D1140" s="3" t="n">
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1141" s="4" t="inlineStr">
+        <is>
+          <t>sz11</t>
+        </is>
+      </c>
+      <c r="C1141" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1141" s="5" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B1142" s="2" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="C1142" s="3" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="D1142" s="3" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B1143" s="4" t="inlineStr">
+        <is>
+          <t>sz01</t>
+        </is>
+      </c>
+      <c r="C1143" s="5" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="D1143" s="5" t="n">
+        <v>-0.04</v>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B1144" s="2" t="inlineStr">
+        <is>
+          <t>sz02</t>
+        </is>
+      </c>
+      <c r="C1144" s="3" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="D1144" s="3" t="n">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B1145" s="4" t="inlineStr">
+        <is>
+          <t>sz03</t>
+        </is>
+      </c>
+      <c r="C1145" s="5" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="D1145" s="5" t="n">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B1146" s="2" t="inlineStr">
+        <is>
+          <t>sz04</t>
+        </is>
+      </c>
+      <c r="C1146" s="3" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="D1146" s="3" t="n">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B1147" s="4" t="inlineStr">
+        <is>
+          <t>sz05</t>
+        </is>
+      </c>
+      <c r="C1147" s="5" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="D1147" s="5" t="n">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B1148" s="2" t="inlineStr">
+        <is>
+          <t>sz06</t>
+        </is>
+      </c>
+      <c r="C1148" s="3" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="D1148" s="3" t="n">
+        <v>-0.04</v>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B1149" s="4" t="inlineStr">
+        <is>
+          <t>sz07</t>
+        </is>
+      </c>
+      <c r="C1149" s="5" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D1149" s="5" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B1150" s="2" t="inlineStr">
+        <is>
+          <t>sz08</t>
+        </is>
+      </c>
+      <c r="C1150" s="3" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="D1150" s="3" t="n">
+        <v>0.58</v>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B1151" s="4" t="inlineStr">
+        <is>
+          <t>sz09</t>
+        </is>
+      </c>
+      <c r="C1151" s="5" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="D1151" s="5" t="n">
+        <v>0.58</v>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B1152" s="2" t="inlineStr">
+        <is>
+          <t>sz10</t>
+        </is>
+      </c>
+      <c r="C1152" s="3" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="D1152" s="3" t="n">
+        <v>0.58</v>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B1153" s="4" t="inlineStr">
+        <is>
+          <t>sz11</t>
+        </is>
+      </c>
+      <c r="C1153" s="5" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="D1153" s="5" t="n">
+        <v>0.58</v>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B1154" s="2" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="C1154" s="3" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="D1154" s="3" t="n">
+        <v>-0.14</v>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B1155" s="4" t="inlineStr">
+        <is>
+          <t>sz01</t>
+        </is>
+      </c>
+      <c r="C1155" s="5" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="D1155" s="5" t="n">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B1156" s="2" t="inlineStr">
+        <is>
+          <t>sz02</t>
+        </is>
+      </c>
+      <c r="C1156" s="3" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="D1156" s="3" t="n">
+        <v>1.24</v>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B1157" s="4" t="inlineStr">
+        <is>
+          <t>sz03</t>
+        </is>
+      </c>
+      <c r="C1157" s="5" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="D1157" s="5" t="n">
+        <v>1.68</v>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B1158" s="2" t="inlineStr">
+        <is>
+          <t>sz04</t>
+        </is>
+      </c>
+      <c r="C1158" s="3" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="D1158" s="3" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B1159" s="4" t="inlineStr">
+        <is>
+          <t>sz05</t>
+        </is>
+      </c>
+      <c r="C1159" s="5" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="D1159" s="5" t="n">
+        <v>1.68</v>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B1160" s="2" t="inlineStr">
+        <is>
+          <t>sz06</t>
+        </is>
+      </c>
+      <c r="C1160" s="3" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="D1160" s="3" t="n">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B1161" s="4" t="inlineStr">
+        <is>
+          <t>sz07</t>
+        </is>
+      </c>
+      <c r="C1161" s="5" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="D1161" s="5" t="n">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B1162" s="2" t="inlineStr">
+        <is>
+          <t>sz08</t>
+        </is>
+      </c>
+      <c r="C1162" s="3" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="D1162" s="3" t="n">
+        <v>1.58</v>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B1163" s="4" t="inlineStr">
+        <is>
+          <t>sz09</t>
+        </is>
+      </c>
+      <c r="C1163" s="5" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="D1163" s="5" t="n">
+        <v>2.32</v>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B1164" s="2" t="inlineStr">
+        <is>
+          <t>sz10</t>
+        </is>
+      </c>
+      <c r="C1164" s="3" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="D1164" s="3" t="n">
+        <v>1.77</v>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B1165" s="4" t="inlineStr">
+        <is>
+          <t>sz11</t>
+        </is>
+      </c>
+      <c r="C1165" s="5" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="D1165" s="5" t="n">
+        <v>2.32</v>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B1166" s="2" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="C1166" s="3" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="D1166" s="3" t="n">
+        <v>-0.41</v>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B1167" s="4" t="inlineStr">
+        <is>
+          <t>sz01</t>
+        </is>
+      </c>
+      <c r="C1167" s="5" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="D1167" s="5" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B1168" s="2" t="inlineStr">
+        <is>
+          <t>sz02</t>
+        </is>
+      </c>
+      <c r="C1168" s="3" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="D1168" s="3" t="n">
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B1169" s="4" t="inlineStr">
+        <is>
+          <t>sz03</t>
+        </is>
+      </c>
+      <c r="C1169" s="5" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="D1169" s="5" t="n">
+        <v>1.53</v>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B1170" s="2" t="inlineStr">
+        <is>
+          <t>sz04</t>
+        </is>
+      </c>
+      <c r="C1170" s="3" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="D1170" s="3" t="n">
+        <v>1.29</v>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B1171" s="4" t="inlineStr">
+        <is>
+          <t>sz05</t>
+        </is>
+      </c>
+      <c r="C1171" s="5" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="D1171" s="5" t="n">
+        <v>1.53</v>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B1172" s="2" t="inlineStr">
+        <is>
+          <t>sz06</t>
+        </is>
+      </c>
+      <c r="C1172" s="3" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="D1172" s="3" t="n">
+        <v>-0.12</v>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B1173" s="4" t="inlineStr">
+        <is>
+          <t>sz07</t>
+        </is>
+      </c>
+      <c r="C1173" s="5" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D1173" s="5" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B1174" s="2" t="inlineStr">
+        <is>
+          <t>sz08</t>
+        </is>
+      </c>
+      <c r="C1174" s="3" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="D1174" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B1175" s="4" t="inlineStr">
+        <is>
+          <t>sz09</t>
+        </is>
+      </c>
+      <c r="C1175" s="5" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="D1175" s="5" t="n">
+        <v>1.77</v>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B1176" s="2" t="inlineStr">
+        <is>
+          <t>sz10</t>
+        </is>
+      </c>
+      <c r="C1176" s="3" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="D1176" s="3" t="n">
+        <v>1.38</v>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B1177" s="4" t="inlineStr">
+        <is>
+          <t>sz11</t>
+        </is>
+      </c>
+      <c r="C1177" s="5" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="D1177" s="5" t="n">
+        <v>2.05</v>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1178" s="2" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="C1178" s="3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="D1178" s="3" t="n">
+        <v>-0.33</v>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1179" s="4" t="inlineStr">
+        <is>
+          <t>sz01</t>
+        </is>
+      </c>
+      <c r="C1179" s="5" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D1179" s="5" t="n">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1180" s="2" t="inlineStr">
+        <is>
+          <t>sz02</t>
+        </is>
+      </c>
+      <c r="C1180" s="3" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="D1180" s="3" t="n">
+        <v>1.01</v>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1181" s="4" t="inlineStr">
+        <is>
+          <t>sz03</t>
+        </is>
+      </c>
+      <c r="C1181" s="5" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="D1181" s="5" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1182" s="2" t="inlineStr">
+        <is>
+          <t>sz04</t>
+        </is>
+      </c>
+      <c r="C1182" s="3" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="D1182" s="3" t="n">
+        <v>1.39</v>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1183" s="4" t="inlineStr">
+        <is>
+          <t>sz05</t>
+        </is>
+      </c>
+      <c r="C1183" s="5" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="D1183" s="5" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1184" s="2" t="inlineStr">
+        <is>
+          <t>sz06</t>
+        </is>
+      </c>
+      <c r="C1184" s="3" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="D1184" s="3" t="n">
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1185" s="4" t="inlineStr">
+        <is>
+          <t>sz07</t>
+        </is>
+      </c>
+      <c r="C1185" s="5" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="D1185" s="5" t="n">
+        <v>0.74</v>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1186" s="2" t="inlineStr">
+        <is>
+          <t>sz08</t>
+        </is>
+      </c>
+      <c r="C1186" s="3" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="D1186" s="3" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1187" s="4" t="inlineStr">
+        <is>
+          <t>sz09</t>
+        </is>
+      </c>
+      <c r="C1187" s="5" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="D1187" s="5" t="n">
+        <v>2.07</v>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1188" s="2" t="inlineStr">
+        <is>
+          <t>sz10</t>
+        </is>
+      </c>
+      <c r="C1188" s="3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D1188" s="3" t="n">
+        <v>1.85</v>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1189" s="4" t="inlineStr">
+        <is>
+          <t>sz11</t>
+        </is>
+      </c>
+      <c r="C1189" s="5" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="D1189" s="5" t="n">
+        <v>2.07</v>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B1190" s="2" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="C1190" s="3" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D1190" s="3" t="n">
+        <v>-0.51</v>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B1191" s="4" t="inlineStr">
+        <is>
+          <t>sz01</t>
+        </is>
+      </c>
+      <c r="C1191" s="5" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D1191" s="5" t="n">
+        <v>0.37</v>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B1192" s="2" t="inlineStr">
+        <is>
+          <t>sz02</t>
+        </is>
+      </c>
+      <c r="C1192" s="3" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="D1192" s="3" t="n">
+        <v>1.13</v>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B1193" s="4" t="inlineStr">
+        <is>
+          <t>sz03</t>
+        </is>
+      </c>
+      <c r="C1193" s="5" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="D1193" s="5" t="n">
+        <v>1.48</v>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B1194" s="2" t="inlineStr">
+        <is>
+          <t>sz04</t>
+        </is>
+      </c>
+      <c r="C1194" s="3" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="D1194" s="3" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B1195" s="4" t="inlineStr">
+        <is>
+          <t>sz05</t>
+        </is>
+      </c>
+      <c r="C1195" s="5" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="D1195" s="5" t="n">
+        <v>1.48</v>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B1196" s="2" t="inlineStr">
+        <is>
+          <t>sz06</t>
+        </is>
+      </c>
+      <c r="C1196" s="3" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="D1196" s="3" t="n">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B1197" s="4" t="inlineStr">
+        <is>
+          <t>sz07</t>
+        </is>
+      </c>
+      <c r="C1197" s="5" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="D1197" s="5" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B1198" s="2" t="inlineStr">
+        <is>
+          <t>sz08</t>
+        </is>
+      </c>
+      <c r="C1198" s="3" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="D1198" s="3" t="n">
+        <v>1.33</v>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B1199" s="4" t="inlineStr">
+        <is>
+          <t>sz09</t>
+        </is>
+      </c>
+      <c r="C1199" s="5" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="D1199" s="5" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B1200" s="2" t="inlineStr">
+        <is>
+          <t>sz10</t>
+        </is>
+      </c>
+      <c r="C1200" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D1200" s="3" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B1201" s="4" t="inlineStr">
+        <is>
+          <t>sz11</t>
+        </is>
+      </c>
+      <c r="C1201" s="5" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="D1201" s="5" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B1202" s="2" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="C1202" s="3" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="D1202" s="3" t="n">
+        <v>-0.45</v>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B1203" s="4" t="inlineStr">
+        <is>
+          <t>sz01</t>
+        </is>
+      </c>
+      <c r="C1203" s="5" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="D1203" s="5" t="n">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B1204" s="2" t="inlineStr">
+        <is>
+          <t>sz02</t>
+        </is>
+      </c>
+      <c r="C1204" s="3" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="D1204" s="3" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B1205" s="4" t="inlineStr">
+        <is>
+          <t>sz03</t>
+        </is>
+      </c>
+      <c r="C1205" s="5" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="D1205" s="5" t="n">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B1206" s="2" t="inlineStr">
+        <is>
+          <t>sz04</t>
+        </is>
+      </c>
+      <c r="C1206" s="3" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="D1206" s="3" t="n">
+        <v>1.12</v>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B1207" s="4" t="inlineStr">
+        <is>
+          <t>sz05</t>
+        </is>
+      </c>
+      <c r="C1207" s="5" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="D1207" s="5" t="n">
+        <v>1.12</v>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B1208" s="2" t="inlineStr">
+        <is>
+          <t>sz06</t>
+        </is>
+      </c>
+      <c r="C1208" s="3" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="D1208" s="3" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B1209" s="4" t="inlineStr">
+        <is>
+          <t>sz07</t>
+        </is>
+      </c>
+      <c r="C1209" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D1209" s="5" t="n">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B1210" s="2" t="inlineStr">
+        <is>
+          <t>sz08</t>
+        </is>
+      </c>
+      <c r="C1210" s="3" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="D1210" s="3" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B1211" s="4" t="inlineStr">
+        <is>
+          <t>sz09</t>
+        </is>
+      </c>
+      <c r="C1211" s="5" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="D1211" s="5" t="n">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B1212" s="2" t="inlineStr">
+        <is>
+          <t>sz10</t>
+        </is>
+      </c>
+      <c r="C1212" s="3" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="D1212" s="3" t="n">
+        <v>1.52</v>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B1213" s="4" t="inlineStr">
+        <is>
+          <t>sz11</t>
+        </is>
+      </c>
+      <c r="C1213" s="5" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="D1213" s="5" t="n">
+        <v>1.52</v>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B1214" s="2" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="C1214" s="3" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="D1214" s="3" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B1215" s="4" t="inlineStr">
+        <is>
+          <t>sz01</t>
+        </is>
+      </c>
+      <c r="C1215" s="5" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="D1215" s="5" t="n">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B1216" s="2" t="inlineStr">
+        <is>
+          <t>sz02</t>
+        </is>
+      </c>
+      <c r="C1216" s="3" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="D1216" s="3" t="n">
+        <v>1.03</v>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B1217" s="4" t="inlineStr">
+        <is>
+          <t>sz03</t>
+        </is>
+      </c>
+      <c r="C1217" s="5" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="D1217" s="5" t="n">
+        <v>1.74</v>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B1218" s="2" t="inlineStr">
+        <is>
+          <t>sz04</t>
+        </is>
+      </c>
+      <c r="C1218" s="3" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="D1218" s="3" t="n">
+        <v>2.89</v>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B1219" s="4" t="inlineStr">
+        <is>
+          <t>sz05</t>
+        </is>
+      </c>
+      <c r="C1219" s="5" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="D1219" s="5" t="n">
+        <v>3.69</v>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B1220" s="2" t="inlineStr">
+        <is>
+          <t>sz06</t>
+        </is>
+      </c>
+      <c r="C1220" s="3" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="D1220" s="3" t="n">
+        <v>-0.02</v>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B1221" s="4" t="inlineStr">
+        <is>
+          <t>sz07</t>
+        </is>
+      </c>
+      <c r="C1221" s="5" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="D1221" s="5" t="n">
+        <v>1.72</v>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B1222" s="2" t="inlineStr">
+        <is>
+          <t>sz08</t>
+        </is>
+      </c>
+      <c r="C1222" s="3" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="D1222" s="3" t="n">
+        <v>1.06</v>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B1223" s="4" t="inlineStr">
+        <is>
+          <t>sz09</t>
+        </is>
+      </c>
+      <c r="C1223" s="5" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="D1223" s="5" t="n">
+        <v>1.73</v>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B1224" s="2" t="inlineStr">
+        <is>
+          <t>sz10</t>
+        </is>
+      </c>
+      <c r="C1224" s="3" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="D1224" s="3" t="n">
+        <v>2.76</v>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B1225" s="4" t="inlineStr">
+        <is>
+          <t>sz11</t>
+        </is>
+      </c>
+      <c r="C1225" s="5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D1225" s="5" t="n">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B1226" s="2" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="C1226" s="3" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="D1226" s="3" t="n">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B1227" s="4" t="inlineStr">
+        <is>
+          <t>sz01</t>
+        </is>
+      </c>
+      <c r="C1227" s="5" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="D1227" s="5" t="n">
+        <v>1.21</v>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B1228" s="2" t="inlineStr">
+        <is>
+          <t>sz02</t>
+        </is>
+      </c>
+      <c r="C1228" s="3" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="D1228" s="3" t="n">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B1229" s="4" t="inlineStr">
+        <is>
+          <t>sz03</t>
+        </is>
+      </c>
+      <c r="C1229" s="5" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="D1229" s="5" t="n">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B1230" s="2" t="inlineStr">
+        <is>
+          <t>sz04</t>
+        </is>
+      </c>
+      <c r="C1230" s="3" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="D1230" s="3" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B1231" s="4" t="inlineStr">
+        <is>
+          <t>sz05</t>
+        </is>
+      </c>
+      <c r="C1231" s="5" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="D1231" s="5" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B1232" s="2" t="inlineStr">
+        <is>
+          <t>sz06</t>
+        </is>
+      </c>
+      <c r="C1232" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1232" s="3" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B1233" s="4" t="inlineStr">
+        <is>
+          <t>sz07</t>
+        </is>
+      </c>
+      <c r="C1233" s="5" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="D1233" s="5" t="n">
+        <v>1.26</v>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B1234" s="2" t="inlineStr">
+        <is>
+          <t>sz08</t>
+        </is>
+      </c>
+      <c r="C1234" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1234" s="3" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B1235" s="4" t="inlineStr">
+        <is>
+          <t>sz09</t>
+        </is>
+      </c>
+      <c r="C1235" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1235" s="5" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B1236" s="2" t="inlineStr">
+        <is>
+          <t>sz10</t>
+        </is>
+      </c>
+      <c r="C1236" s="3" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="D1236" s="3" t="n">
+        <v>1.77</v>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B1237" s="4" t="inlineStr">
+        <is>
+          <t>sz11</t>
+        </is>
+      </c>
+      <c r="C1237" s="5" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="D1237" s="5" t="n">
+        <v>1.77</v>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B1238" s="2" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="C1238" s="3" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="D1238" s="3" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B1239" s="4" t="inlineStr">
+        <is>
+          <t>sz01</t>
+        </is>
+      </c>
+      <c r="C1239" s="5" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="D1239" s="5" t="n">
+        <v>0.63</v>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B1240" s="2" t="inlineStr">
+        <is>
+          <t>sz02</t>
+        </is>
+      </c>
+      <c r="C1240" s="3" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="D1240" s="3" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B1241" s="4" t="inlineStr">
+        <is>
+          <t>sz03</t>
+        </is>
+      </c>
+      <c r="C1241" s="5" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="D1241" s="5" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B1242" s="2" t="inlineStr">
+        <is>
+          <t>sz04</t>
+        </is>
+      </c>
+      <c r="C1242" s="3" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="D1242" s="3" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B1243" s="4" t="inlineStr">
+        <is>
+          <t>sz05</t>
+        </is>
+      </c>
+      <c r="C1243" s="5" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D1243" s="5" t="n">
+        <v>2.21</v>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B1244" s="2" t="inlineStr">
+        <is>
+          <t>sz06</t>
+        </is>
+      </c>
+      <c r="C1244" s="3" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="D1244" s="3" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B1245" s="4" t="inlineStr">
+        <is>
+          <t>sz07</t>
+        </is>
+      </c>
+      <c r="C1245" s="5" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="D1245" s="5" t="n">
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B1246" s="2" t="inlineStr">
+        <is>
+          <t>sz08</t>
+        </is>
+      </c>
+      <c r="C1246" s="3" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="D1246" s="3" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B1247" s="4" t="inlineStr">
+        <is>
+          <t>sz09</t>
+        </is>
+      </c>
+      <c r="C1247" s="5" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="D1247" s="5" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B1248" s="2" t="inlineStr">
+        <is>
+          <t>sz10</t>
+        </is>
+      </c>
+      <c r="C1248" s="3" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="D1248" s="3" t="n">
+        <v>1.55</v>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B1249" s="4" t="inlineStr">
+        <is>
+          <t>sz11</t>
+        </is>
+      </c>
+      <c r="C1249" s="5" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="D1249" s="5" t="n">
+        <v>2.3</v>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B1250" s="2" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="C1250" s="3" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="D1250" s="3" t="n">
+        <v>-0.48</v>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B1251" s="4" t="inlineStr">
+        <is>
+          <t>sz01</t>
+        </is>
+      </c>
+      <c r="C1251" s="5" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="D1251" s="5" t="n">
+        <v>0.54</v>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B1252" s="2" t="inlineStr">
+        <is>
+          <t>sz02</t>
+        </is>
+      </c>
+      <c r="C1252" s="3" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="D1252" s="3" t="n">
+        <v>-0.01</v>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B1253" s="4" t="inlineStr">
+        <is>
+          <t>sz03</t>
+        </is>
+      </c>
+      <c r="C1253" s="5" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="D1253" s="5" t="n">
+        <v>-0.01</v>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B1254" s="2" t="inlineStr">
+        <is>
+          <t>sz04</t>
+        </is>
+      </c>
+      <c r="C1254" s="3" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="D1254" s="3" t="n">
+        <v>1.18</v>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B1255" s="4" t="inlineStr">
+        <is>
+          <t>sz05</t>
+        </is>
+      </c>
+      <c r="C1255" s="5" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="D1255" s="5" t="n">
+        <v>1.18</v>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B1256" s="2" t="inlineStr">
+        <is>
+          <t>sz06</t>
+        </is>
+      </c>
+      <c r="C1256" s="3" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="D1256" s="3" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B1257" s="4" t="inlineStr">
+        <is>
+          <t>sz07</t>
+        </is>
+      </c>
+      <c r="C1257" s="5" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="D1257" s="5" t="n">
+        <v>0.77</v>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B1258" s="2" t="inlineStr">
+        <is>
+          <t>sz08</t>
+        </is>
+      </c>
+      <c r="C1258" s="3" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="D1258" s="3" t="n">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B1259" s="4" t="inlineStr">
+        <is>
+          <t>sz09</t>
+        </is>
+      </c>
+      <c r="C1259" s="5" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="D1259" s="5" t="n">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B1260" s="2" t="inlineStr">
+        <is>
+          <t>sz10</t>
+        </is>
+      </c>
+      <c r="C1260" s="3" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="D1260" s="3" t="n">
+        <v>1.66</v>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B1261" s="4" t="inlineStr">
+        <is>
+          <t>sz11</t>
+        </is>
+      </c>
+      <c r="C1261" s="5" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="D1261" s="5" t="n">
+        <v>1.66</v>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B1262" s="2" t="inlineStr">
+        <is>
+          <t>real</t>
+        </is>
+      </c>
+      <c r="C1262" s="3" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="D1262" s="3" t="n">
+        <v>-0.13</v>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B1263" s="4" t="inlineStr">
+        <is>
+          <t>sz01</t>
+        </is>
+      </c>
+      <c r="C1263" s="5" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="D1263" s="5" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B1264" s="2" t="inlineStr">
+        <is>
+          <t>sz02</t>
+        </is>
+      </c>
+      <c r="C1264" s="3" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="D1264" s="3" t="n">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B1265" s="4" t="inlineStr">
+        <is>
+          <t>sz03</t>
+        </is>
+      </c>
+      <c r="C1265" s="5" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="D1265" s="5" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B1266" s="2" t="inlineStr">
+        <is>
+          <t>sz04</t>
+        </is>
+      </c>
+      <c r="C1266" s="3" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="D1266" s="3" t="n">
+        <v>1.15</v>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B1267" s="4" t="inlineStr">
+        <is>
+          <t>sz05</t>
+        </is>
+      </c>
+      <c r="C1267" s="5" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="D1267" s="5" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B1268" s="2" t="inlineStr">
+        <is>
+          <t>sz06</t>
+        </is>
+      </c>
+      <c r="C1268" s="3" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="D1268" s="3" t="n">
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B1269" s="4" t="inlineStr">
+        <is>
+          <t>sz07</t>
+        </is>
+      </c>
+      <c r="C1269" s="5" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="D1269" s="5" t="n">
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B1270" s="2" t="inlineStr">
+        <is>
+          <t>sz08</t>
+        </is>
+      </c>
+      <c r="C1270" s="3" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="D1270" s="3" t="n">
+        <v>1.13</v>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B1271" s="4" t="inlineStr">
+        <is>
+          <t>sz09</t>
+        </is>
+      </c>
+      <c r="C1271" s="5" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="D1271" s="5" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B1272" s="2" t="inlineStr">
+        <is>
+          <t>sz10</t>
+        </is>
+      </c>
+      <c r="C1272" s="3" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="D1272" s="3" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B1273" s="4" t="inlineStr">
+        <is>
+          <t>sz11</t>
+        </is>
+      </c>
+      <c r="C1273" s="5" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="D1273" s="5" t="n">
+        <v>2.01</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D1081"/>
+  <autoFilter ref="A1:D1273"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>